<commit_message>
featured images were added
</commit_message>
<xml_diff>
--- a/content/publication/mypubs_2025_07.xlsx
+++ b/content/publication/mypubs_2025_07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliguner/Documents/Rsites/aliguner/content/publication/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B068971-58E2-7C48-8D34-9CD30C0FCF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F57D56-47B4-D24A-8EAD-1CE654D88F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="21020" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="920">
   <si>
     <t>value</t>
   </si>
@@ -2733,9 +2733,6 @@
     </r>
   </si>
   <si>
-    <t>10.4174/astr.2025.108.2.86.</t>
-  </si>
-  <si>
     <t>Ann Surg Treat Res. 2025 Feb;108(2):86-92.</t>
   </si>
   <si>
@@ -2828,12 +2825,30 @@
   <si>
     <t>AI</t>
   </si>
+  <si>
+    <t>TASMAN Collaborative,</t>
+  </si>
+  <si>
+    <t>OGAAO Collaborative,</t>
+  </si>
+  <si>
+    <t>GlobalSurg Collaborative,</t>
+  </si>
+  <si>
+    <t>EuroSurg Collaborative,</t>
+  </si>
+  <si>
+    <t>OGAA Collaborative,</t>
+  </si>
+  <si>
+    <t>10.4174/astr.2025.108.2.86</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2902,12 +2917,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="27"/>
-      <color rgb="FF333333"/>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
-    </font>
-    <font>
       <i/>
       <sz val="17"/>
       <color rgb="FF2A2A2A"/>
@@ -2955,7 +2964,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3332,10 +3341,10 @@
         <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>525</v>
+        <v>918</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="G2" t="s">
         <v>852</v>
@@ -3356,7 +3365,7 @@
         <v>853</v>
       </c>
       <c r="M2" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N2" t="s">
         <v>677</v>
@@ -3376,7 +3385,7 @@
         <v>679</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>854</v>
@@ -3394,10 +3403,10 @@
         <v>683</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N3" t="s">
         <v>684</v>
@@ -3476,7 +3485,7 @@
         <v>858</v>
       </c>
       <c r="M5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N5" t="s">
         <v>698</v>
@@ -3493,7 +3502,7 @@
         <v>111</v>
       </c>
       <c r="D6" t="s">
-        <v>340</v>
+        <v>917</v>
       </c>
       <c r="E6" t="s">
         <v>700</v>
@@ -3517,7 +3526,7 @@
         <v>861</v>
       </c>
       <c r="M6" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N6" t="s">
         <v>703</v>
@@ -3534,10 +3543,10 @@
         <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>321</v>
+        <v>916</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>862</v>
@@ -3558,7 +3567,7 @@
         <v>863</v>
       </c>
       <c r="M7" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N7" t="s">
         <v>709</v>
@@ -3596,7 +3605,7 @@
         <v>864</v>
       </c>
       <c r="M8" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="N8" t="s">
         <v>715</v>
@@ -3669,7 +3678,7 @@
         <v>869</v>
       </c>
       <c r="M10" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N10" t="s">
         <v>728</v>
@@ -3710,7 +3719,7 @@
         <v>871</v>
       </c>
       <c r="M11" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N11" t="s">
         <v>733</v>
@@ -3751,7 +3760,7 @@
         <v>873</v>
       </c>
       <c r="M12" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N12" t="s">
         <v>739</v>
@@ -3792,7 +3801,7 @@
         <v>875</v>
       </c>
       <c r="M13" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N13" t="s">
         <v>745</v>
@@ -3833,7 +3842,7 @@
         <v>876</v>
       </c>
       <c r="M14" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N14" t="s">
         <v>751</v>
@@ -3874,13 +3883,13 @@
         <v>878</v>
       </c>
       <c r="M15" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N15" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="86" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="30" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>758</v>
       </c>
@@ -3894,7 +3903,7 @@
         <v>759</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>880</v>
@@ -3915,7 +3924,7 @@
         <v>881</v>
       </c>
       <c r="M16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N16" t="s">
         <v>764</v>
@@ -3956,7 +3965,7 @@
         <v>882</v>
       </c>
       <c r="M17" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="N17" t="s">
         <v>771</v>
@@ -3973,7 +3982,7 @@
         <v>123</v>
       </c>
       <c r="D18" t="s">
-        <v>773</v>
+        <v>914</v>
       </c>
       <c r="E18" t="s">
         <v>774</v>
@@ -3997,7 +4006,7 @@
         <v>885</v>
       </c>
       <c r="M18" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N18" t="s">
         <v>777</v>
@@ -4071,7 +4080,7 @@
       </c>
       <c r="L20" s="4"/>
       <c r="M20" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N20" t="s">
         <v>789</v>
@@ -4094,7 +4103,7 @@
         <v>792</v>
       </c>
       <c r="G21" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="I21" t="s">
         <v>793</v>
@@ -4106,7 +4115,7 @@
         <v>795</v>
       </c>
       <c r="L21" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="N21" t="s">
         <v>796</v>
@@ -4129,7 +4138,7 @@
         <v>799</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H22" s="2">
         <v>38504597</v>
@@ -4144,7 +4153,7 @@
         <v>801</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="N22" t="s">
         <v>802</v>
@@ -4167,7 +4176,7 @@
         <v>806</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="H23" s="2">
         <v>40554350</v>
@@ -4183,7 +4192,7 @@
       </c>
       <c r="L23" s="4"/>
       <c r="M23" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N23" t="s">
         <v>810</v>
@@ -4206,7 +4215,7 @@
         <v>813</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H24" s="2">
         <v>40481693</v>
@@ -4221,7 +4230,7 @@
         <v>815</v>
       </c>
       <c r="L24" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="N24" t="s">
         <v>816</v>
@@ -4244,7 +4253,7 @@
         <v>819</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="H25" s="2">
         <v>40472748</v>
@@ -4256,10 +4265,10 @@
         <v>821</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="M25" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="N25" t="s">
         <v>822</v>
@@ -4276,13 +4285,13 @@
         <v>131</v>
       </c>
       <c r="D26" t="s">
-        <v>824</v>
+        <v>915</v>
       </c>
       <c r="E26" t="s">
         <v>825</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="H26" s="2">
         <v>40405118</v>
@@ -4297,10 +4306,10 @@
         <v>827</v>
       </c>
       <c r="L26" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="M26" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N26" t="s">
         <v>828</v>
@@ -4332,7 +4341,7 @@
         <v>833</v>
       </c>
       <c r="M27" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N27" t="s">
         <v>834</v>
@@ -4352,10 +4361,10 @@
         <v>836</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="H28" s="2">
         <v>40067192</v>
@@ -4370,10 +4379,10 @@
         <v>839</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="M28" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N28" t="s">
         <v>840</v>
@@ -4393,10 +4402,10 @@
         <v>842</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>899</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>890</v>
+        <v>898</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>919</v>
       </c>
       <c r="H29" s="2">
         <v>39944923</v>
@@ -4411,10 +4420,10 @@
         <v>846</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="M29" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N29" t="s">
         <v>847</v>
@@ -4427,6 +4436,7 @@
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" display="https://doi.org/10.1093/jbcr/irz004" xr:uid="{CE9346B4-E304-B346-8776-2E86767C3F2E}"/>
     <hyperlink ref="G20" r:id="rId2" display="https://doi.org/10.1093/bjs/znae129" xr:uid="{3F1FA75D-AC69-5F4F-82CC-6731FC91D456}"/>
+    <hyperlink ref="G29" r:id="rId3" display="https://doi.org/10.4174/astr.2025.108.2.86" xr:uid="{2D1179AB-741B-3844-8474-B26AB08B9F15}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>